<commit_message>
added some links in new links
</commit_message>
<xml_diff>
--- a/Advanced_Architectures_and_deployment/Designing_custom_architectures/newlinks.xlsx
+++ b/Advanced_Architectures_and_deployment/Designing_custom_architectures/newlinks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bosch-my.sharepoint.com/personal/csu5kor_bosch_com/Documents/Coursera/pytorch_training/pytorch_training/Advanced_Architectures_and_deployment/Designing_custom_architectures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_F25DC773A252ABDACC104836D9DF74F65ADE5902" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1770C5D1-0F50-48D9-8CFA-7CE06C93F79D}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="11_F25DC773A252ABDACC104836D9DF74F65ADE5902" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42EAA44A-4C5B-4B4C-83CB-EE94FB8F9BB1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>sl.no</t>
   </si>
@@ -46,6 +46,27 @@
   </si>
   <si>
     <t>https://amaarora.github.io/posts/2020-08-02-densenets.html</t>
+  </si>
+  <si>
+    <t>https://cs231n.github.io/convolutional-networks/#conv</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=pYaAMx_GfH0</t>
+  </si>
+  <si>
+    <t>https://lilianweng.github.io/posts/2021-07-11-diffusion-models/</t>
+  </si>
+  <si>
+    <t>convolution concepts</t>
+  </si>
+  <si>
+    <t>saliency maps</t>
+  </si>
+  <si>
+    <t>diffusion models</t>
+  </si>
+  <si>
+    <t>https://huggingface.co/docs/diffusers/index</t>
   </si>
 </sst>
 </file>
@@ -363,13 +384,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="50.88671875" customWidth="1"/>
+    <col min="2" max="2" width="65.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -377,7 +398,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -385,7 +406,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -393,7 +414,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -401,7 +422,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -409,12 +430,56 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>